<commit_message>
Préparation de la release 2.0.0
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> d4ed3164270a66d70a40771285f0b07cc4661d83
</commit_message>
<xml_diff>
--- a/nr-release-2.0.0/ig/StructureDefinition-TDEBundleResultatReponseRechercheTraces.xlsx
+++ b/nr-release-2.0.0/ig/StructureDefinition-TDEBundleResultatReponseRechercheTraces.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0-ballot</t>
+    <t>2.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -45,7 +45,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-13T15:21:42+00:00</t>
+    <t>2026-03-13T15:25:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>